<commit_message>
CTDC updates for Input files
</commit_message>
<xml_diff>
--- a/InputFiles/CTDC/TC01_CTDC_AnatomCollecSite-AbdomWall.xlsx
+++ b/InputFiles/CTDC/TC01_CTDC_AnatomCollecSite-AbdomWall.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\epishinavv\git\Commons_Automation\InputFiles\CTDC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/epishinavv/git/Commons_Automation/InputFiles/CTDC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4CED9FE-9129-42F4-B1FF-70CC65C9120D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0876345E-58A0-E844-8540-5D26041474A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8362173B-D28C-47E7-8626-98E16101E601}"/>
+    <workbookView xWindow="6960" yWindow="780" windowWidth="29040" windowHeight="15720" xr2:uid="{8362173B-D28C-47E7-8626-98E16101E601}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -109,7 +109,101 @@
     AND bio.anatomical_collection_site = 'Abdominal Wall';</t>
   </si>
   <si>
+    <t>SELECT
+    prt.participant_id AS "Participant ID",
+    dgn.ctep_disease_term AS "Diagnosis",
+    demo.age_at_enrollment AS "Age",
+    demo.sex AS "Sex",
+    demo.race AS "Race",
+    demo.ethnicity AS "Ethnicity",
+    exp.carcinogen_exposure AS "Carcinogen Exposure",
+    REPLACE(
+        GROUP_CONCAT(
+            DISTINCT
+            UPPER(SUBSTR(LOWER(tgt.targeted_therapy), 1, 1)) ||
+            SUBSTR(LOWER(tgt.targeted_therapy), 2)
+        ),
+        ',',
+        ', '
+    ) AS "Targeted Therapy"
+FROM 
+    df_study std
+LEFT JOIN df_participant prt 
+    ON std.study_short_name = prt."study.study_short_name"
+LEFT JOIN df_diagnosis dgn 
+    ON prt.participant_id = dgn."participant.participant_id"
+LEFT JOIN df_demographic demo 
+    ON prt.participant_id = demo."participant.participant_id"
+LEFT JOIN df_exposure exp 
+    ON prt.participant_id = exp."participant.participant_id"
+LEFT JOIN df_targeted_therapy tgt 
+    ON prt.participant_id = tgt."participant.participant_id"
+LEFT JOIN df_non_targeted_therapy ntt 
+    ON prt.participant_id = ntt."participant.participant_id"
+LEFT JOIN df_participant_status pst 
+    ON prt.participant_id = pst."participant.participant_id"
+LEFT JOIN df_biospecimen bio 
+    ON prt.participant_id = bio."participant.participant_id"
+LEFT JOIN df_file fil 
+    ON prt.participant_id = fil."participant.participant_id"
+WHERE 
+    std.study_id = 'NCT04314401'
+    AND bio.anatomical_collection_site = 'Abdominal Wall'
+GROUP BY
+    prt.participant_id,
+    dgn.ctep_disease_term,
+    demo.age_at_enrollment,
+    demo.sex,
+    demo.race,
+    demo.ethnicity,
+    exp.carcinogen_exposure
+LIMIT 100;</t>
+  </si>
+  <si>
     <t>SELECT DISTINCT
+    prt.participant_id AS "Participant ID",
+    dgn.ctep_disease_term AS "Diagnosis",
+    dgn.primary_disease_site AS "Primary Site",
+    bio.specimen_record_id AS "Specimen Record ID",
+    bio.anatomical_collection_site AS "Anatomical Collection Site",
+    bio.tissue_category AS "Tissue Category",
+    bio.assessment_timepoint AS "Collection Timepoint"
+FROM 
+    df_study std
+LEFT JOIN 
+    df_participant prt 
+        ON std.study_short_name = prt."study.study_short_name"
+LEFT JOIN 
+    df_diagnosis dgn 
+        ON prt.participant_id = dgn."participant.participant_id"
+LEFT JOIN 
+    df_demographic demo 
+        ON prt.participant_id = demo."participant.participant_id"
+LEFT JOIN 
+    df_exposure exp 
+        ON prt.participant_id = exp."participant.participant_id"
+LEFT JOIN 
+    df_targeted_therapy tgt 
+        ON prt.participant_id = tgt."participant.participant_id"
+LEFT JOIN 
+    df_non_targeted_therapy ntt 
+        ON prt.participant_id = ntt."participant.participant_id"
+LEFT JOIN 
+    df_participant_status pst 
+        ON prt.participant_id = pst."participant.participant_id"
+LEFT JOIN 
+    df_biospecimen bio 
+        ON prt.participant_id = bio."participant.participant_id"
+LEFT JOIN 
+    df_file fil 
+        ON prt.participant_id = fil."participant.participant_id"
+WHERE 
+    std.study_id = 'NCT04314401' AND bio.anatomical_collection_site = 'Abdominal Wall'
+LIMIT 100;</t>
+  </si>
+  <si>
+    <t>SELECT DISTINCT
+std.study_accession as "Study Accession",
     fil.data_file_name AS "File Name",
     LOWER(fil.data_file_format) AS "Format",
     fil.data_file_type AS "File Type",
@@ -172,107 +266,21 @@
     AND fil.data_file_name IS NOT NULL
 LIMIT 100;</t>
   </si>
-  <si>
-    <t>SELECT
-    prt.participant_id AS "Participant ID",
-    dgn.ctep_disease_term AS "Diagnosis",
-    demo.age_at_enrollment AS "Age",
-    demo.sex AS "Sex",
-    demo.race AS "Race",
-    demo.ethnicity AS "Ethnicity",
-    exp.carcinogen_exposure AS "Carcinogen Exposure",
-    REPLACE(
-        GROUP_CONCAT(
-            DISTINCT
-            UPPER(SUBSTR(LOWER(tgt.targeted_therapy), 1, 1)) ||
-            SUBSTR(LOWER(tgt.targeted_therapy), 2)
-        ),
-        ',',
-        ', '
-    ) AS "Targeted Therapy"
-FROM 
-    df_study std
-LEFT JOIN df_participant prt 
-    ON std.study_short_name = prt."study.study_short_name"
-LEFT JOIN df_diagnosis dgn 
-    ON prt.participant_id = dgn."participant.participant_id"
-LEFT JOIN df_demographic demo 
-    ON prt.participant_id = demo."participant.participant_id"
-LEFT JOIN df_exposure exp 
-    ON prt.participant_id = exp."participant.participant_id"
-LEFT JOIN df_targeted_therapy tgt 
-    ON prt.participant_id = tgt."participant.participant_id"
-LEFT JOIN df_non_targeted_therapy ntt 
-    ON prt.participant_id = ntt."participant.participant_id"
-LEFT JOIN df_participant_status pst 
-    ON prt.participant_id = pst."participant.participant_id"
-LEFT JOIN df_biospecimen bio 
-    ON prt.participant_id = bio."participant.participant_id"
-LEFT JOIN df_file fil 
-    ON prt.participant_id = fil."participant.participant_id"
-WHERE 
-    std.study_id = 'NCT04314401'
-    AND bio.anatomical_collection_site = 'Abdominal Wall'
-GROUP BY
-    prt.participant_id,
-    dgn.ctep_disease_term,
-    demo.age_at_enrollment,
-    demo.sex,
-    demo.race,
-    demo.ethnicity,
-    exp.carcinogen_exposure
-LIMIT 100;</t>
-  </si>
-  <si>
-    <t>SELECT DISTINCT
-    prt.participant_id AS "Participant ID",
-    dgn.ctep_disease_term AS "Diagnosis",
-    dgn.primary_disease_site AS "Primary Site",
-    bio.specimen_record_id AS "Specimen Record ID",
-    bio.anatomical_collection_site AS "Anatomical Collection Site",
-    bio.tissue_category AS "Tissue Category",
-    bio.assessment_timepoint AS "Collection Timepoint"
-FROM 
-    df_study std
-LEFT JOIN 
-    df_participant prt 
-        ON std.study_short_name = prt."study.study_short_name"
-LEFT JOIN 
-    df_diagnosis dgn 
-        ON prt.participant_id = dgn."participant.participant_id"
-LEFT JOIN 
-    df_demographic demo 
-        ON prt.participant_id = demo."participant.participant_id"
-LEFT JOIN 
-    df_exposure exp 
-        ON prt.participant_id = exp."participant.participant_id"
-LEFT JOIN 
-    df_targeted_therapy tgt 
-        ON prt.participant_id = tgt."participant.participant_id"
-LEFT JOIN 
-    df_non_targeted_therapy ntt 
-        ON prt.participant_id = ntt."participant.participant_id"
-LEFT JOIN 
-    df_participant_status pst 
-        ON prt.participant_id = pst."participant.participant_id"
-LEFT JOIN 
-    df_biospecimen bio 
-        ON prt.participant_id = bio."participant.participant_id"
-LEFT JOIN 
-    df_file fil 
-        ON prt.participant_id = fil."participant.participant_id"
-WHERE 
-    std.study_id = 'NCT04314401' AND bio.anatomical_collection_site = 'Abdominal Wall'
-LIMIT 100;</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -325,11 +333,14 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -654,16 +665,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C538400-E87C-4027-A918-A51DB80B3430}">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="75.77734375" customWidth="1"/>
-    <col min="3" max="3" width="60.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="45.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="75.83203125" customWidth="1"/>
+    <col min="3" max="3" width="60.83203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="45.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="46.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>2</v>
       </c>
@@ -680,12 +691,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="297" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" ht="297" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>10</v>
@@ -697,28 +708,28 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="372" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="372" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>11</v>
+      <c r="B4" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="C4" s="2"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="C5" s="1"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="4" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>

</xml_diff>